<commit_message>
feat: add listing workflow and tarot cards SKU
</commit_message>
<xml_diff>
--- a/src/listing-system/商品数据.xlsx
+++ b/src/listing-system/商品数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,13 +906,75 @@
           <t>133181542011</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>2026-03-16 22:37:26</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02-2603-0001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Oracle Tarot Cards - Japanese Language Edition Fortune Telling Deck 78 Cards</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>&lt;h2&gt;Oracle Tarot Cards&lt;/h2&gt;&lt;p&gt;Beautiful 78-card tarot deck in Japanese. Perfect for fortune telling and spiritual guidance.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>45112</v>
+      </c>
+      <c r="E7" t="n">
+        <v>68.42</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>OTC-2603-001</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Does not apply</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="M7" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="N7" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="O7" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add Amazon images to 02-2603-0001
</commit_message>
<xml_diff>
--- a/src/listing-system/商品数据.xlsx
+++ b/src/listing-system/商品数据.xlsx
@@ -942,7 +942,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/71ozeGv+hfL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71fgX-axY-L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/61pUFBnLanL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/716uLrks40L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71K04bKnf4L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71jro2gfJ8L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/61t1CI+e9zL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71y1BvEQbjL._AC_SL1400_.jpg</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Generic</t>
@@ -970,11 +974,6 @@
       <c r="O7" t="n">
         <v>3</v>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: optimize 02-2603-0001 tarot cards listing data
- Remove HOBO products (keep only 02-2603-0001)
- Correct category: 35837 (Collectible Wiccan & Pagan Tarot Cards)
- Full SEO-optimized English title and description
- Correct brand and MPN from Amazon
</commit_message>
<xml_diff>
--- a/src/listing-system/商品数据.xlsx
+++ b/src/listing-system/商品数据.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,27 +521,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HOBO-5Y-2026</t>
+          <t>02-2603-0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hobonichi 5-Year Techo Gift Edition 2026-2030 haconiwa Limited</t>
+          <t>Japanese Mythology Divine Oracle Cards - 36 Deities Tarot Deck - Spiritual Divination Fortune Telling</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>&lt;h2&gt;Hobonichi 5-Year Techo&lt;/h2&gt;&lt;p&gt;Premium planner 2026-2030.&lt;/p&gt;</t>
+          <t>&lt;h2&gt;Japanese Mythology Divine Oracle Cards&lt;/h2&gt;
+&lt;p&gt;&lt;strong&gt;36-Card Deck | Japanese Edition | Authentic&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;Experience the ancient wisdom of Japanese mythology with this beautifully crafted Divine Oracle Cards deck. Featuring 36 deity cards inspired by Shinto and Japanese folklore traditions.&lt;/p&gt;
+&lt;h3&gt;Product Features:&lt;/h3&gt;
+&lt;ul&gt;
+&lt;li&gt;&lt;strong&gt;36 unique cards&lt;/strong&gt; depicting ancient Japanese deities and mythological figures&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Language:&lt;/strong&gt; Japanese (original edition)&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Perfect for:&lt;/strong&gt; Tarot readings, spiritual guidance, meditation, divination practice&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Suitable for:&lt;/strong&gt; Both beginners and experienced tarot readers&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Compact size:&lt;/strong&gt; Easy to shuffle and handle&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Includes:&lt;/strong&gt; Complete 36-card oracle deck&lt;/li&gt;
+&lt;/ul&gt;
+&lt;h3&gt;Specifications:&lt;/h3&gt;
+&lt;ul&gt;
+&lt;li&gt;&lt;strong&gt;Card Count:&lt;/strong&gt; 36 cards&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Condition:&lt;/strong&gt; Brand New&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Authentic:&lt;/strong&gt; Genuine imported product&lt;/li&gt;
+&lt;/ul&gt;
+&lt;h3&gt;Usage:&lt;/h3&gt;
+&lt;p&gt;Ideal for daily spiritual guidance, meditation practice, fortune telling sessions, and exploring Japanese cultural wisdom through divination.&lt;/p&gt;
+&lt;p&gt;&lt;em&gt;Add this authentic Japanese oracle deck to your collection today!&lt;/em&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>45112</v>
+        <v>35837</v>
       </c>
       <c r="E2" t="n">
-        <v>49.99</v>
+        <v>68.42</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -550,17 +570,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://example.com/image1.jpg,https://example.com/image2.jpg</t>
+          <t>https://m.media-amazon.com/images/I/71ozeGv+hfL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71fgX-axY-L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/61pUFBnLanL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/716uLrks40L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71K04bKnf4L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71jro2gfJ8L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/61t1CI+e9zL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71y1BvEQbjL._AC_SL1400_.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Hobonichi</t>
+          <t>LC Infinity Lulu Couture</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>T26-HC-001</t>
+          <t>01-36-088</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -569,409 +589,15 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.33</v>
+        <v>0.16</v>
       </c>
       <c r="M2" t="n">
-        <v>15.3</v>
+        <v>12.7</v>
       </c>
       <c r="N2" t="n">
-        <v>11.3</v>
+        <v>7.6</v>
       </c>
       <c r="O2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="n">
-        <v>133163244011</v>
-      </c>
-      <c r="R2" t="n">
-        <v>397720980732</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>2026-03-16 21:10:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HOBO-WEEKS-2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Hobonichi Techo Weeks 2026 Sneaker Navy x Orange</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Compact weekly planner with Tomoe River paper.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>45112</v>
-      </c>
-      <c r="E3" t="n">
-        <v>29.99</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://example.com/weeks1.jpg</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Hobonichi</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>W26-SN-001</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Does not apply</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M3" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="N3" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="n">
-        <v>133163277011</v>
-      </c>
-      <c r="R3" t="n">
-        <v>397720981176</v>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>2026-03-16 21:10:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>HOBO-DIARY-2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Hobonichi Techo 2026 Diary A6 Size Cousin Cover</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Authentic Japanese Hobonichi Techo 2026 daily planner. A6 size with cousin fabric cover. Features Tomoe River paper, time stamps, and monthly spreads. Perfect for bullet journaling and daily planning.</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>45112</v>
-      </c>
-      <c r="E4" t="n">
-        <v>39.99</v>
-      </c>
-      <c r="F4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://i.ebayimg.com/images/g/abc123/s-l1600.jpg</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Hobonichi</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>1012603083</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Does not apply</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M4" t="n">
-        <v>21</v>
-      </c>
-      <c r="N4" t="n">
-        <v>14</v>
-      </c>
-      <c r="O4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q4" t="n">
-        <v>133163292011</v>
-      </c>
-      <c r="R4" t="n">
-        <v>397720981516</v>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>2026-03-16 21:10:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HOBO-MARINE-2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hobonichi Techo 2026 Marine Blue Cover with Gold Thread</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Limited edition Hobonichi Techo 2026 in marine blue with elegant gold thread stitching. A6 size, daily planner format.</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>45112</v>
-      </c>
-      <c r="E5" t="n">
-        <v>44.99</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://i.ebayimg.com/images/g/xyz789/s-l1600.jpg</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Hobonichi</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>1012603099</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Does not apply</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M5" t="n">
-        <v>21</v>
-      </c>
-      <c r="N5" t="n">
-        <v>14</v>
-      </c>
-      <c r="O5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>133163309011</v>
-      </c>
-      <c r="R5" t="n">
-        <v>397720981846</v>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>2026-03-16 21:10:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>HOBO-TEST-2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Hobonichi Techo 2026 Test Edition - For Review</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>This is a test listing for the review web interface. Please review before publishing.</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>45112</v>
-      </c>
-      <c r="E6" t="n">
-        <v>99.98999999999999</v>
-      </c>
-      <c r="F6" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://httpbin.org/image</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Hobonichi</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>TEST-001</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Does not apply</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M6" t="n">
-        <v>21</v>
-      </c>
-      <c r="N6" t="n">
-        <v>14</v>
-      </c>
-      <c r="O6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>133181542011</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>2026-03-16 22:37:26</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>02-2603-0001</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Oracle Tarot Cards - Japanese Language Edition Fortune Telling Deck 78 Cards</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>&lt;h2&gt;Oracle Tarot Cards&lt;/h2&gt;&lt;p&gt;Beautiful 78-card tarot deck in Japanese. Perfect for fortune telling and spiritual guidance.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>45112</v>
-      </c>
-      <c r="E7" t="n">
-        <v>68.42</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://m.media-amazon.com/images/I/71ozeGv+hfL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71fgX-axY-L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/61pUFBnLanL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/716uLrks40L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71K04bKnf4L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71jro2gfJ8L._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/61t1CI+e9zL._AC_SL1400_.jpg,https://m.media-amazon.com/images/I/71y1BvEQbjL._AC_SL1400_.jpg</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>OTC-2603-001</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Does not apply</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="M7" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="N7" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="O7" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>